<commit_message>
fix: horário de escalonamento
</commit_message>
<xml_diff>
--- a/CheckLists de autoria/Checklists/3 - 1 NC resolvida e outra escalonada.xlsx
+++ b/CheckLists de autoria/Checklists/3 - 1 NC resolvida e outra escalonada.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\PlanoGarantiaQualidade\CheckLists de autoria\Checklists\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{000DD989-02F4-4509-9D3F-CC772BECFFF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{035E5931-8D67-4301-9D14-275225353168}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Checklist - Auditoria" sheetId="1" r:id="rId1"/>
@@ -563,18 +563,8 @@
     <xf numFmtId="22" fontId="10" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="4" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -584,7 +574,17 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="4" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -889,19 +889,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="40" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
-      <c r="G1" s="32"/>
-      <c r="H1" s="32"/>
-      <c r="I1" s="32"/>
-      <c r="J1" s="32"/>
-      <c r="K1" s="32"/>
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="40"/>
+      <c r="I1" s="40"/>
+      <c r="J1" s="40"/>
+      <c r="K1" s="40"/>
     </row>
     <row r="2" spans="1:11" ht="48" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
@@ -939,19 +939,19 @@
       </c>
     </row>
     <row r="3" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="33" t="s">
+      <c r="A3" s="41" t="s">
         <v>43</v>
       </c>
-      <c r="B3" s="33"/>
-      <c r="C3" s="33"/>
-      <c r="D3" s="33"/>
-      <c r="E3" s="33"/>
-      <c r="F3" s="33"/>
-      <c r="G3" s="33"/>
-      <c r="H3" s="33"/>
-      <c r="I3" s="33"/>
-      <c r="J3" s="33"/>
-      <c r="K3" s="33"/>
+      <c r="B3" s="41"/>
+      <c r="C3" s="41"/>
+      <c r="D3" s="41"/>
+      <c r="E3" s="41"/>
+      <c r="F3" s="41"/>
+      <c r="G3" s="41"/>
+      <c r="H3" s="41"/>
+      <c r="I3" s="41"/>
+      <c r="J3" s="41"/>
+      <c r="K3" s="41"/>
     </row>
     <row r="4" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3">
@@ -1076,19 +1076,19 @@
       <c r="K8" s="4"/>
     </row>
     <row r="9" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="33" t="s">
+      <c r="A9" s="41" t="s">
         <v>44</v>
       </c>
-      <c r="B9" s="33"/>
-      <c r="C9" s="33"/>
-      <c r="D9" s="33"/>
-      <c r="E9" s="33"/>
-      <c r="F9" s="33"/>
-      <c r="G9" s="33"/>
-      <c r="H9" s="33"/>
-      <c r="I9" s="33"/>
-      <c r="J9" s="33"/>
-      <c r="K9" s="33"/>
+      <c r="B9" s="41"/>
+      <c r="C9" s="41"/>
+      <c r="D9" s="41"/>
+      <c r="E9" s="41"/>
+      <c r="F9" s="41"/>
+      <c r="G9" s="41"/>
+      <c r="H9" s="41"/>
+      <c r="I9" s="41"/>
+      <c r="J9" s="41"/>
+      <c r="K9" s="41"/>
     </row>
     <row r="10" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3">
@@ -1201,19 +1201,19 @@
       <c r="K14" s="4"/>
     </row>
     <row r="15" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="33" t="s">
+      <c r="A15" s="41" t="s">
         <v>50</v>
       </c>
-      <c r="B15" s="33"/>
-      <c r="C15" s="33"/>
-      <c r="D15" s="33"/>
-      <c r="E15" s="33"/>
-      <c r="F15" s="33"/>
-      <c r="G15" s="33"/>
-      <c r="H15" s="33"/>
-      <c r="I15" s="33"/>
-      <c r="J15" s="33"/>
-      <c r="K15" s="33"/>
+      <c r="B15" s="41"/>
+      <c r="C15" s="41"/>
+      <c r="D15" s="41"/>
+      <c r="E15" s="41"/>
+      <c r="F15" s="41"/>
+      <c r="G15" s="41"/>
+      <c r="H15" s="41"/>
+      <c r="I15" s="41"/>
+      <c r="J15" s="41"/>
+      <c r="K15" s="41"/>
     </row>
     <row r="16" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="3">
@@ -1459,7 +1459,7 @@
         <v>46269.463194444441</v>
       </c>
       <c r="I27" s="31">
-        <v>46269.421527777777</v>
+        <v>46269.428472222222</v>
       </c>
       <c r="J27" s="24"/>
       <c r="K27" s="26" t="s">
@@ -1545,81 +1545,81 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="37" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
-      <c r="F1" s="34"/>
-      <c r="G1" s="34"/>
+      <c r="B1" s="37"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="37"/>
+      <c r="F1" s="37"/>
+      <c r="G1" s="37"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="35" t="s">
+      <c r="A2" s="38" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="35"/>
-      <c r="C2" s="35"/>
-      <c r="D2" s="35"/>
-      <c r="E2" s="35"/>
-      <c r="F2" s="35"/>
-      <c r="G2" s="35"/>
+      <c r="B2" s="38"/>
+      <c r="C2" s="38"/>
+      <c r="D2" s="38"/>
+      <c r="E2" s="38"/>
+      <c r="F2" s="38"/>
+      <c r="G2" s="38"/>
     </row>
     <row r="4" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="B4" s="36" t="s">
+      <c r="B4" s="33" t="s">
         <v>76</v>
       </c>
-      <c r="C4" s="36"/>
-      <c r="D4" s="36"/>
-      <c r="E4" s="36"/>
+      <c r="C4" s="33"/>
+      <c r="D4" s="33"/>
+      <c r="E4" s="33"/>
     </row>
     <row r="5" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="36" t="s">
+      <c r="B5" s="33" t="s">
         <v>77</v>
       </c>
-      <c r="C5" s="36"/>
-      <c r="D5" s="36"/>
-      <c r="E5" s="36"/>
+      <c r="C5" s="33"/>
+      <c r="D5" s="33"/>
+      <c r="E5" s="33"/>
     </row>
     <row r="6" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="37">
+      <c r="B6" s="39">
         <v>46269</v>
       </c>
-      <c r="C6" s="37"/>
-      <c r="D6" s="37"/>
-      <c r="E6" s="37"/>
+      <c r="C6" s="39"/>
+      <c r="D6" s="39"/>
+      <c r="E6" s="39"/>
     </row>
     <row r="7" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B7" s="36" t="s">
+      <c r="B7" s="33" t="s">
         <v>75</v>
       </c>
-      <c r="C7" s="36"/>
-      <c r="D7" s="36"/>
-      <c r="E7" s="36"/>
+      <c r="C7" s="33"/>
+      <c r="D7" s="33"/>
+      <c r="E7" s="33"/>
     </row>
     <row r="8" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="36" t="s">
+      <c r="B8" s="33" t="s">
         <v>18</v>
       </c>
-      <c r="C8" s="36"/>
-      <c r="D8" s="36"/>
-      <c r="E8" s="36"/>
+      <c r="C8" s="33"/>
+      <c r="D8" s="33"/>
+      <c r="E8" s="33"/>
     </row>
     <row r="10" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="7" t="s">
@@ -1667,23 +1667,23 @@
       </c>
     </row>
     <row r="16" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="34" t="s">
         <v>24</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="34"/>
     </row>
     <row r="17" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39">
+      <c r="A17" s="35">
         <f>IFERROR(B11/(B10-B13),0)</f>
         <v>0.9</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="35"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A19" s="40" t="s">
+      <c r="A19" s="36" t="s">
         <v>25</v>
       </c>
-      <c r="B19" s="40"/>
+      <c r="B19" s="36"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" s="9" t="s">
@@ -1770,70 +1770,80 @@
       <c r="A31" s="7"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A32" s="41"/>
-      <c r="B32" s="41"/>
-      <c r="C32" s="41"/>
-      <c r="D32" s="41"/>
-      <c r="E32" s="41"/>
-      <c r="F32" s="41"/>
-      <c r="G32" s="41"/>
+      <c r="A32" s="32"/>
+      <c r="B32" s="32"/>
+      <c r="C32" s="32"/>
+      <c r="D32" s="32"/>
+      <c r="E32" s="32"/>
+      <c r="F32" s="32"/>
+      <c r="G32" s="32"/>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A33" s="41"/>
-      <c r="B33" s="41"/>
-      <c r="C33" s="41"/>
-      <c r="D33" s="41"/>
-      <c r="E33" s="41"/>
-      <c r="F33" s="41"/>
-      <c r="G33" s="41"/>
+      <c r="A33" s="32"/>
+      <c r="B33" s="32"/>
+      <c r="C33" s="32"/>
+      <c r="D33" s="32"/>
+      <c r="E33" s="32"/>
+      <c r="F33" s="32"/>
+      <c r="G33" s="32"/>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A34" s="41"/>
-      <c r="B34" s="41"/>
-      <c r="C34" s="41"/>
-      <c r="D34" s="41"/>
-      <c r="E34" s="41"/>
-      <c r="F34" s="41"/>
-      <c r="G34" s="41"/>
+      <c r="A34" s="32"/>
+      <c r="B34" s="32"/>
+      <c r="C34" s="32"/>
+      <c r="D34" s="32"/>
+      <c r="E34" s="32"/>
+      <c r="F34" s="32"/>
+      <c r="G34" s="32"/>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A35" s="41"/>
-      <c r="B35" s="41"/>
-      <c r="C35" s="41"/>
-      <c r="D35" s="41"/>
-      <c r="E35" s="41"/>
-      <c r="F35" s="41"/>
-      <c r="G35" s="41"/>
+      <c r="A35" s="32"/>
+      <c r="B35" s="32"/>
+      <c r="C35" s="32"/>
+      <c r="D35" s="32"/>
+      <c r="E35" s="32"/>
+      <c r="F35" s="32"/>
+      <c r="G35" s="32"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A36" s="41"/>
-      <c r="B36" s="41"/>
-      <c r="C36" s="41"/>
-      <c r="D36" s="41"/>
-      <c r="E36" s="41"/>
-      <c r="F36" s="41"/>
-      <c r="G36" s="41"/>
+      <c r="A36" s="32"/>
+      <c r="B36" s="32"/>
+      <c r="C36" s="32"/>
+      <c r="D36" s="32"/>
+      <c r="E36" s="32"/>
+      <c r="F36" s="32"/>
+      <c r="G36" s="32"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A37" s="41"/>
-      <c r="B37" s="41"/>
-      <c r="C37" s="41"/>
-      <c r="D37" s="41"/>
-      <c r="E37" s="41"/>
-      <c r="F37" s="41"/>
-      <c r="G37" s="41"/>
+      <c r="A37" s="32"/>
+      <c r="B37" s="32"/>
+      <c r="C37" s="32"/>
+      <c r="D37" s="32"/>
+      <c r="E37" s="32"/>
+      <c r="F37" s="32"/>
+      <c r="G37" s="32"/>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A38" s="41"/>
-      <c r="B38" s="41"/>
-      <c r="C38" s="41"/>
-      <c r="D38" s="41"/>
-      <c r="E38" s="41"/>
-      <c r="F38" s="41"/>
-      <c r="G38" s="41"/>
+      <c r="A38" s="32"/>
+      <c r="B38" s="32"/>
+      <c r="C38" s="32"/>
+      <c r="D38" s="32"/>
+      <c r="E38" s="32"/>
+      <c r="F38" s="32"/>
+      <c r="G38" s="32"/>
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="B4:E4"/>
+    <mergeCell ref="B5:E5"/>
+    <mergeCell ref="B6:E6"/>
+    <mergeCell ref="B7:E7"/>
+    <mergeCell ref="B8:E8"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="A19:B19"/>
     <mergeCell ref="A37:G37"/>
     <mergeCell ref="A38:G38"/>
     <mergeCell ref="A32:G32"/>
@@ -1841,16 +1851,6 @@
     <mergeCell ref="A34:G34"/>
     <mergeCell ref="A35:G35"/>
     <mergeCell ref="A36:G36"/>
-    <mergeCell ref="B7:E7"/>
-    <mergeCell ref="B8:E8"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="A19:B19"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="B4:E4"/>
-    <mergeCell ref="B5:E5"/>
-    <mergeCell ref="B6:E6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>